<commit_message>
Revise size-series strategy: kW pages merge into converted kVA pages; small-kVA pruning option
kVA-kW Matrix now maps each kW page to its converted 301 target (kW/0.8
rounded up, never same-number), per-page checklist and recommendations
updated, sub-50kVA pages flagged as prune candidates pending client floor
decision.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199Ec3JvGkM5VeF3Edd8KdB
</commit_message>
<xml_diff>
--- a/Solent-Power-SEO-Plan-Content-Research.xlsx
+++ b/Solent-Power-SEO-Plan-Content-Research.xlsx
@@ -20,15 +20,15 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Recommendations'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Recommendations'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Keyword Universe'!$A$1:$J$196</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Clusters'!$A$1:$G$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cannibalisation Validation'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Commercial Architecture'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Informational Architecture'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'kVA-kW Matrix'!$A$1:$F$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'kVA-kW Matrix'!$A$1:$H$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Per-Page Checklist'!$A$1:$H$524</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Linking &amp; Global Rules'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Linking &amp; Global Rules'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -789,8 +789,20 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>kW-&gt;kVA merge &amp; pruning</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>The kW-series merge and any small-size pruning are ONE sanctioned consolidation batch: single 301s to the converted-rating kVA page (never same-number), kW equivalent added to title + H2 BEFORE the redirects go live, then the URL graph freezes for a quarter. Do not stage it page-by-page over weeks - Google re-evaluates once.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -801,10 +813,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -974,122 +986,147 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>kVA series cleanup: categories own size terms; retitle every product to its model term; fold ≤25kW pages into kVA twins; cross-link remaining twins; ADD large-size pages 350/600/700/800/900/1250/1500/2000kVA.</t>
+          <t>Single kVA size series (client-agreed): retire ALL kW pages via one 301 each to the kVA page covering the converted rating (kW÷0.8 rounded up — 200kW→250kVA, 100kW→150kVA; never same-number). kVA titles carry the kW equivalent + an H2 conversion note, added BEFORE redirects go live. Categories own size terms; retitle every product to its model term; ADD 70/90/110/350/900/1250/1500/2000/2500kVA.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Products outrank own categories (30/45/60/80/250/300kVA — validated); 800kVA (150/mo) = the onboarding's explicit best-fit signal with a weak, stale SERP; 110kVA has 866 impressions and no page.</t>
+          <t>Products outrank own categories (validated); one URL provably ranks for both rating families (Solent's Pramac GSW250P '200kW 250kVA' product does today); kW series = 266 clicks/90d, 60% from sub-ICP 10-20kW pages; 800kVA+ ladder = the onboarding's best-fit deal signal.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Size demand consolidates onto categories; the large-generator ladder matches the actual sales sweet spot.</t>
+          <t>One coherent size ladder matched to how the industry specs machines; short-term dip on kW terms, recovery via 301 equity at KD 0.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>P3 · Weeks 8-12</t>
+          <t>P3 · CLIENT DECISION</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Informational link engine: optimise the transfer-switch guide (10k impressions pos 9), oil guide (25k impressions), sizing guide (merge duplicate), kVA-vs-kW chart; every guide links down to its commercial page with exact anchors.</t>
+          <t>Set the small-generator pruning floor. Proposal: prune below 50kVA — 301 the 10/20/25/30/40kVA categories + their kW feeders into /diesel-generators/, retire or noindex the ~68 sub-50kVA products. Softer option: keep them live but remove from nav/homepage/link spine (no equity, no investment).</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>The blog already earns most non-checker visibility (628k impressions across 95 articles); its equity currently goes nowhere commercial.</t>
+          <t>Sub-50kVA estate currently earns ~600 clicks/90d (146 category + ~170 small-kW + 287 product clicks) — over half of all commercial clicks, none of it the 800kVA+/continuity ICP. Pruning is a positioning play: it changes what Google (and AI answers) think the site IS, at the cost of a visible traffic drop in reports.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Cheapest ranking lever: internal equity flows to the money pages.</t>
+          <t>Client must confirm the smallest generator they still want to sell/service before this batch ships. Traffic will drop; qualified relevance rises.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>P4 · Quarter 2</t>
+          <t>P3 · Weeks 8-12</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Brand consolidation (/brand/ + /generator-sales/{x}-generators/ → /brands/{x}/), sector pages (healthcare + HTM 06-01 guide, data centres, manufacturing), BESS merge.</t>
+          <t>Informational link engine: optimise the transfer-switch guide (10k impressions pos 9), oil guide (25k impressions), sizing guide (merge duplicate), kVA-vs-kW chart; every guide links down to its commercial page with exact anchors.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>himoinsa n=2 URLs; htm 06-01 = 150/mo at £4.50 CPC with KD 0; sectors are the ICP door-openers (near-zero volume, maximum fit).</t>
+          <t>The blog already earns most non-checker visibility (628k impressions across 95 articles); its equity currently goes nowhere commercial.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Entity clarity per brand; sales-enablement pages that convert consultants/M&amp;E.</t>
+          <t>Cheapest ranking lever: internal equity flows to the money pages.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Always</t>
+          <t>P4 · Quarter 2</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>FREEZE the URL graph after each consolidation batch; re-pull GSC cannibalisation evidence at weeks 6-8 per phase. Success metric: one URL per query cluster; servicing CTR &gt;1%.</t>
+          <t>Brand consolidation (/brand/ + /generator-sales/{x}-generators/ → /brands/{x}/), sector pages (healthcare + HTM 06-01 guide, data centres, manufacturing), BESS merge.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Redirect churn is how sites lose head terms; Google needs a stable graph to re-evaluate.</t>
+          <t>himoinsa n=2 URLs; htm 06-01 = 150/mo at £4.50 CPC with KD 0; sectors are the ICP door-openers (near-zero volume, maximum fit).</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Measurable, reversible-free rollout.</t>
+          <t>Entity clarity per brand; sales-enablement pages that convert consultants/M&amp;E.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>FREEZE the URL graph after each consolidation batch; re-pull GSC cannibalisation evidence at weeks 6-8 per phase. Success metric: one URL per query cluster; servicing CTR &gt;1%.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Redirect churn is how sites lose head terms; Google needs a stable graph to re-evaluate.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Measurable, reversible-free rollout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Hygiene</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Password-protect staging2 (live, crawlable, noindexed today); keep filter URLs noindexed; fix HTML-entity sitemap encoding if present; no other technical emergencies found (no penalty signature; growth plateau matches structural diagnosis).</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>staging2 serves 200s with x-robots noindex; filter params crawlable but not indexed (SERPAPI-verified).</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Risk removal, not rankings.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9574,7 +9611,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>KEEP both series (SERPs differ) but disambiguate: kVA page titles = standby/prime rating + 'kVA', kW titles = kW with kVA equivalent named; hard cross-link each twin pair (100kW ↔ 125kVA); small sizes where Google maps kW→kVA parent (≤25kW) get kW folded into the kVA page with a 301.</t>
+          <t>MERGE (client-agreed): one kVA-only series. Every kW page 301s to the kVA page covering its converted rating (kVA = kW ÷ 0.8, rounded UP to the next page — e.g. 200kW→250kVA, 100kW→150kVA; NEVER same-number, 200kVA ≠ 200kW). Each kVA page carries the kW equivalent in the title ('250kVA Diesel Generators (200kW)') and an H2 with the conversion. Evidence one URL can rank for both families: Solent's own Pramac GSW250P '200kW 250kVA' product already ranks in both. Known trade: kW pages earn ~89 clicks/mo (60% from sub-ICP 10-20kW) — expect a dip and recovery via 301 equity at KD 0.</t>
         </is>
       </c>
     </row>
@@ -10234,7 +10271,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Category owns size term (validated). ADD missing ICP sizes: 350/600/700/800/900/1250/1500/2000kVA — '800 kva generator' (150/mo) SERP is stale &amp; weak = open. These are the deal-size terms (800kVA+ = onboarding's best-fit signal).</t>
+          <t>Category owns size term (validated). kVA becomes the ONLY size series (kW pages merge in — see Matrix tab). Titles carry the kW equivalent: '{N}kVA Diesel Generators ({kW}kW) | UK Stock'. H2 states the conversion. ADD missing sizes: 70/90/110/350/900/1250/1500/2000/2500kVA (600/700/800 already exist) — the 800kVA+ ladder is the deal-size signal. CLIENT DECISION: pruning floor — proposed 50kVA; pages below it are prune candidates (see Matrix + Recommendations).</t>
         </is>
       </c>
     </row>
@@ -10251,15 +10288,19 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>EXISTS ×21 - disambiguate</t>
+          <t>MERGE - 301 all (P3)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>'{N}kw generator' where SERP distinct</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>(none - series retired)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>kW terms captured on kVA pages via title/H2 equivalents</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Size category</t>
@@ -10267,7 +10308,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Keep where SERP differs (validated ≥50kW); fold ≤25kW pages into kVA twins (301) where Google maps kw→kva parent. Cross-link every twin pair.</t>
+          <t>Client-agreed merge. Each kW page 301s ONCE to the kVA page ≥ its converted rating (kW÷0.8, round up): 40kW→50kVA · 50kW→70kVA · 60kW→80kVA · 70kW→90kVA · 80kW→100kVA · 90/100kW→150kVA · 150kW→200kVA · 200kW→250kVA · 250kW→350kVA · 300kW→400kVA · 400kW→500kVA · 500kW→700kVA · 600kW→800kVA · 800kW→1000kVA · 900kW→1250kVA. 10-30kW pages: if the &lt;50kVA floor is pruned they 301 to /diesel-generators/; else to 20/25/40kVA per Matrix. One batch, then freeze.</t>
         </is>
       </c>
     </row>
@@ -11303,21 +11344,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="64" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>kVA size</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -11327,386 +11370,493 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>kVA page exists</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+          <t>kVA page</t>
+        </is>
+      </c>
+      <c r="D1" s="1">
+        <f> kW rating</f>
+        <v/>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>kW page exists</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>kW vol/mo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>kW page exists</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>kW page 301 target</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
+      <c r="A2" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="n">
         <v>700</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>8kW</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client to confirm smallest size they want to sell/service). If pruned: this page + its kW feeders 301 to /diesel-generators/. If kept: absorbs its kW feeders per mapping, demoted from nav/link spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>FOLD /generators/10kw/ into /generators/10kva/ twin (301) — Google maps small kW to kVA parents</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>16kW</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>10kW, 15kW</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>210</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 10kW, 15kW</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client to confirm smallest size they want to sell/service). If pruned: this page + its kW feeders 301 to /diesel-generators/. If kept: absorbs its kW feeders per mapping, demoted from nav/link spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>20kW</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>20kW</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 20kW</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client to confirm smallest size they want to sell/service). If pruned: this page + its kW feeders 301 to /diesel-generators/. If kept: absorbs its kW feeders per mapping, demoted from nav/link spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>24kW</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client to confirm smallest size they want to sell/service). If pruned: this page + its kW feeders 301 to /diesel-generators/. If kept: absorbs its kW feeders per mapping, demoted from nav/link spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>32kW</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>25kW, 30kW</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 25kW, 30kW</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client to confirm smallest size they want to sell/service). If pruned: this page + its kW feeders 301 to /diesel-generators/. If kept: absorbs its kW feeders per mapping, demoted from nav/link spine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>FOLD /generators/15kw/ into /generators/15kva/ twin (301) — Google maps small kW to kVA parents</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>40kW</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>40kW</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 40kW</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 40kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B8" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>48kW</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; title/H2 state the kW equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="B9" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>56kW</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>50kW</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 50kW</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL; absorbs 50kW on creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>FOLD /generators/20kw/ into /generators/25kva/ twin (301) — Google maps small kW to kVA parents</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>64kW</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>60kW</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 60kW</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 60kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>72kW</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>70kW</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 70kW</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL; absorbs 70kW on creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B12" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>80kW</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>80kW</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 80kW</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 80kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>88kW</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>FOLD /generators/25kw/ into /generators/25kva/ twin (301) — Google maps small kW to kVA parents</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>120kW</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>90kW, 100kW</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 90kW, 100kW</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 90kW, 100kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>200</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/70kva/ — demand with no page</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/90kva/ — demand with no page</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/110kva/ — demand with no page</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
       </c>
       <c r="B15" s="2" t="n">
         <v>200</v>
@@ -11716,51 +11866,67 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>160kW</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>150kW</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 150kW</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 150kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>200kW</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>200kW</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 200kW</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 200kW; add kW equivalent to title + H2 BEFORE redirecting</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
+      <c r="A17" s="2" t="n">
+        <v>300</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>80</v>
@@ -11770,211 +11936,277 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>240kW</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; title/H2 state the kW equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>280kW</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>250kW</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 250kW</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder); absorbs 250kW on creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>320kW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>300kW</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 300kW</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 300kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>400kW</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>400kW</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 400kW</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 400kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>480kW</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; title/H2 state the kW equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>560kW</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>500kW</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 500kW</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 500kW; add kW equivalent to title + H2 BEFORE redirecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>90</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/350kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>450</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Category owns the term; products link up with exact anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="n">
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>640kW</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>600kW</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 600kW</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 600kW; add kW equivalent to title + H2 BEFORE redirecting</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Category owns the term; products link up with exact anchor</t>
+      <c r="A24" s="4" t="n">
+        <v>900</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>720kW</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>800</t>
-        </is>
+      <c r="A25" s="2" t="n">
+        <v>1000</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>150</v>
@@ -11984,178 +12216,182 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>800kW</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Keep both; disambiguate titles (state kW + kVA equivalent) and cross-link the twin pair</t>
+          <t>800kW</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>absorbs 800kW</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>kVA page owns the size; 301 in 800kW; add kW equivalent to title + H2 BEFORE redirecting</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
+      <c r="A26" s="4" t="n">
+        <v>1250</v>
       </c>
       <c r="B26" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>1000kW</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>900kW</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/900kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>absorbs 900kW</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder); absorbs 900kW on creation</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="n">
+      <c r="A27" s="4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>1200kW</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>1600kW</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B29" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Category owns the term; products link up with exact anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>1250</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/1250kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>1500</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>50</v>
-      </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="n"/>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>2000kW</t>
+        </is>
+      </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/1500kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>ADD PAGE — demand with no URL · ICP anchor size (800kVA+ ladder)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/2000kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>2500</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>ADD /generators/2500kva/ — demand with no page · ICP anchor size (800kVA+ = best-fit signal)</t>
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>MAPPING RULE: a kW page 301s to the kVA page whose rating ≥ kW÷0.8 (200kW→250kVA, 100kW→150kVA). NEVER same-number (200kVA=160kW, not 200kW). Titles: '{N}kVA Diesel Generators ({kW}kW)'. One batch, then freeze.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F31"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15065,7 +15301,7 @@
       <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client decision). If pruned: 301 to /diesel-generators/ with its kW feeders. If kept: merchandised title incl kW equivalent, demoted from nav/link spine.</t>
         </is>
       </c>
     </row>
@@ -15125,7 +15361,7 @@
       <c r="G98" s="2" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/20kva/ (converted rating, kW÷0.8 rounded up). Add '10kW' to that page's title/H2 BEFORE redirecting. NOTE: below proposed 50kVA pruning floor — if pruning is confirmed, 301 to /diesel-generators/ instead.</t>
         </is>
       </c>
     </row>
@@ -15155,7 +15391,7 @@
       <c r="G99" s="2" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client decision). If pruned: 301 to /diesel-generators/ with its kW feeders. If kept: merchandised title incl kW equivalent, demoted from nav/link spine. Absorbs 10kW, 15kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15283,7 +15519,7 @@
       <c r="G103" s="2" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '500kva generator' term: title '500kVA Diesel Generators (400kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 400kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15313,7 +15549,7 @@
       <c r="G104" s="2" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '1000kva generator' term: title '1000kVA Diesel Generators (800kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 800kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15373,7 +15609,7 @@
       <c r="G106" s="2" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '150kva generator' term: title '150kVA Diesel Generators (120kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 90kW, 100kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15403,7 +15639,7 @@
       <c r="G107" s="2" t="inlineStr"/>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '100kva generator' term: title '100kVA Diesel Generators (80kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 80kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15433,7 +15669,7 @@
       <c r="G108" s="2" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '200kva generator' term: title '200kVA Diesel Generators (160kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 150kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15629,7 +15865,7 @@
       <c r="G114" s="2" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/25kva/ (converted rating, kW÷0.8 rounded up). Add '20kW' to that page's title/H2 BEFORE redirecting. NOTE: below proposed 50kVA pruning floor — if pruning is confirmed, 301 to /diesel-generators/ instead.</t>
         </is>
       </c>
     </row>
@@ -15723,7 +15959,7 @@
       <c r="G117" s="2" t="inlineStr"/>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '250kva generator' term: title '250kVA Diesel Generators (200kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 200kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15787,7 +16023,7 @@
       <c r="G119" s="2" t="inlineStr"/>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/150kva/ (converted rating, kW÷0.8 rounded up). Add '100kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -15817,7 +16053,7 @@
       <c r="G120" s="2" t="inlineStr"/>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '80kva generator' term: title '80kVA Diesel Generators (64kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 60kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15881,7 +16117,7 @@
       <c r="G122" s="2" t="inlineStr"/>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client decision). If pruned: 301 to /diesel-generators/ with its kW feeders. If kept: merchandised title incl kW equivalent, demoted from nav/link spine. Absorbs 25kW, 30kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -15911,7 +16147,7 @@
       <c r="G123" s="2" t="inlineStr"/>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '60kva generator' term: title '60kVA Diesel Generators (48kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell.</t>
         </is>
       </c>
     </row>
@@ -15941,7 +16177,7 @@
       <c r="G124" s="2" t="inlineStr"/>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '400kva generator' term: title '400kVA Diesel Generators (320kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 300kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -16069,7 +16305,7 @@
       <c r="G128" s="2" t="inlineStr"/>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client decision). If pruned: 301 to /diesel-generators/ with its kW feeders. If kept: merchandised title incl kW equivalent, demoted from nav/link spine. Absorbs 20kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -16099,7 +16335,7 @@
       <c r="G129" s="2" t="inlineStr"/>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '300kva generator' term: title '300kVA Diesel Generators (240kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell.</t>
         </is>
       </c>
     </row>
@@ -16223,7 +16459,7 @@
       <c r="G133" s="2" t="inlineStr"/>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/20kva/ (converted rating, kW÷0.8 rounded up). Add '15kW' to that page's title/H2 BEFORE redirecting. NOTE: below proposed 50kVA pruning floor — if pruning is confirmed, 301 to /diesel-generators/ instead.</t>
         </is>
       </c>
     </row>
@@ -16347,7 +16583,7 @@
       <c r="G137" s="2" t="inlineStr"/>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/700kva/ (converted rating, kW÷0.8 rounded up). Add '500kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -16479,7 +16715,7 @@
       <c r="G141" s="2" t="inlineStr"/>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '50kva generator' term: title '50kVA Diesel Generators (40kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 40kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -16663,7 +16899,7 @@
       <c r="G147" s="2" t="inlineStr"/>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '800kva generator' term: title '800kVA Diesel Generators (640kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 600kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -16693,7 +16929,7 @@
       <c r="G148" s="2" t="inlineStr"/>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/50kva/ (converted rating, kW÷0.8 rounded up). Add '40kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -16825,7 +17061,7 @@
       <c r="G152" s="2" t="inlineStr"/>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '700kva generator' term: title '700kVA Diesel Generators (560kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell. Absorbs 500kW (301 in).</t>
         </is>
       </c>
     </row>
@@ -16889,7 +17125,7 @@
       <c r="G154" s="2" t="inlineStr"/>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/400kva/ (converted rating, kW÷0.8 rounded up). Add '300kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -16919,7 +17155,7 @@
       <c r="G155" s="2" t="inlineStr"/>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/40kva/ (converted rating, kW÷0.8 rounded up). Add '30kW' to that page's title/H2 BEFORE redirecting. NOTE: below proposed 50kVA pruning floor — if pruning is confirmed, 301 to /diesel-generators/ instead.</t>
         </is>
       </c>
     </row>
@@ -16949,7 +17185,7 @@
       <c r="G156" s="2" t="inlineStr"/>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>Own the '600kva generator' term: title '600kVA Diesel Generators (480kW) | UK Stock, from £X', H2 conversion note, link adjacent sizes + top 3 models + servicing cross-sell.</t>
         </is>
       </c>
     </row>
@@ -17077,7 +17313,7 @@
       <c r="G160" s="2" t="inlineStr"/>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/250kva/ (converted rating, kW÷0.8 rounded up). Add '200kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -17243,7 +17479,7 @@
       <c r="G165" s="2" t="inlineStr"/>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/70kva/ (converted rating, kW÷0.8 rounded up). Add '50kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17645,7 @@
       <c r="G170" s="2" t="inlineStr"/>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/500kva/ (converted rating, kW÷0.8 rounded up). Add '400kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -17439,7 +17675,7 @@
       <c r="G171" s="2" t="inlineStr"/>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/1000kva/ (converted rating, kW÷0.8 rounded up). Add '800kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -17703,7 +17939,7 @@
       <c r="G179" s="2" t="inlineStr"/>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/100kva/ (converted rating, kW÷0.8 rounded up). Add '80kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -17933,7 +18169,7 @@
       <c r="G186" s="2" t="inlineStr"/>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>Own the '{N}kva generator' term: merchandised title ('UK Stock, from £X'), intro copy w/ standby/prime ratings, link twin kW page + adjacent sizes + top 3 models (text links) + servicing cross-sell.</t>
+          <t>PRUNE CANDIDATE (below proposed 50kVA floor — client decision). If pruned: 301 to /diesel-generators/ with its kW feeders. If kept: merchandised title incl kW equivalent, demoted from nav/link spine.</t>
         </is>
       </c>
     </row>
@@ -18065,7 +18301,7 @@
       <c r="G190" s="2" t="inlineStr"/>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/40kva/ (converted rating, kW÷0.8 rounded up). Add '25kW' to that page's title/H2 BEFORE redirecting. NOTE: below proposed 50kVA pruning floor — if pruning is confirmed, 301 to /diesel-generators/ instead.</t>
         </is>
       </c>
     </row>
@@ -18197,7 +18433,7 @@
       <c r="G194" s="2" t="inlineStr"/>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/350kva/ (converted rating, kW÷0.8 rounded up). Add '250kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -18295,7 +18531,7 @@
       <c r="G197" s="2" t="inlineStr"/>
       <c r="H197" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/90kva/ (converted rating, kW÷0.8 rounded up). Add '70kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -18427,7 +18663,7 @@
       <c r="G201" s="2" t="inlineStr"/>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/200kva/ (converted rating, kW÷0.8 rounded up). Add '150kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -18593,7 +18829,7 @@
       <c r="G206" s="2" t="inlineStr"/>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/800kva/ (converted rating, kW÷0.8 rounded up). Add '600kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -19537,7 +19773,7 @@
       <c r="G234" s="2" t="inlineStr"/>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/80kva/ (converted rating, kW÷0.8 rounded up). Add '60kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -19567,7 +19803,7 @@
       <c r="G235" s="2" t="inlineStr"/>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/150kva/ (converted rating, kW÷0.8 rounded up). Add '90kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>
@@ -21259,7 +21495,7 @@
       <c r="G285" s="2" t="inlineStr"/>
       <c r="H285" s="2" t="inlineStr">
         <is>
-          <t>Disambiguate from kVA twin: title states kW + kVA equivalent; cross-link twin; ≤25kW pages: fold into kVA twin (301) per matrix tab.</t>
+          <t>RETIRE (client-agreed): 301 once to /generators/1250kva/ (converted rating, kW÷0.8 rounded up). Add '900kW' to that page's title/H2 BEFORE redirecting.</t>
         </is>
       </c>
     </row>

</xml_diff>